<commit_message>
fix(seo): configure canonical and sitemaps for krilliononline and playblockblastunblocked
</commit_message>
<xml_diff>
--- a/游戏关键词台账.xlsx
+++ b/游戏关键词台账.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="游戏好词挖掘_2026-10-22" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="游戏好词挖掘_2026-10-23" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +46,18 @@
       <name val="Microsoft YaHei"/>
       <b val="1"/>
       <color rgb="009C6500"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00008000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FF8C00"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -100,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -116,6 +129,24 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -482,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -871,6 +902,1188 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>minute cryptic unlimited</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>每日字谜/填字无限制网页练习站</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Trends +5950% (主词 minute cryptic 月搜 246k, KD 14)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>SERP 极其脆弱：前5充斥 TikTok 视频、官方使用条款页(/tcs)及会员收费页，无真正免费无限练习站</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>模式与付费墙缺口 (官站锁历史题/限制每日1题，急需免费无限与归档)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>立项 (强推)</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>打造 Minute Cryptic Unlimited 纯静态练习器，含提示天梯与历史题库，直击 246k 泛搜索与 4.4k 精准需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>krillion unlimited</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>逆向冷门词汇海洋下潜答题游戏</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Trends +37200% 暴增 (主词 krillion 月搜 165k, KD 0, CPC $12.30)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>SERP 前5为聚合目录和 Instagram Reel，官方每日仅限7题，玩家对连续练习/无限制下潜需求激增</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>内容供给缺口 (无限题库与移动端体验)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>立项 (高价值)</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>开发 Krillion Unlimited 无限下潜模拟器，依托高 CPC ($12.3) 实现 AdSense 超额收益</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>poople game</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>趣味四字母变词成语梯网页游戏</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>12100</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Trends +9350% 爆发 (主词 poople 月搜 165k, KD 0)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>SERP #1 为 ResetEra 论坛讨论帖，#2 为 YouTube 视频，原生独立站极弱，极易反超霸屏</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>形态缺口 (缺乏极致轻量、零加载延迟的免安装 Web 应用)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>立项 (极易开发)</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>四字母 Word Ladder 算法简单，1天内即可用纯原生 JS 产出高颜值、高幽默感的极简即玩站</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>minecraftle unlimited</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>我的世界 3x3 合成配方推理解谜</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>110</v>
+      </c>
+      <c r="D12" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Trends +50% 稳增 (主词 minecraftle 月搜 18.1k, KD 25)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>前排由 zachmanson 与 mcdle 分割，竞争初具雏形但长尾需求仍有空间</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>功能整合缺口 (配方合成+怪物图鉴多合一)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>观察</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>体量适中但已有成熟独立站在打，建议作为 GameHubs 站内二级栏目，暂不单独起独立域名</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>关键词 (Keyword)</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>意图归属 (Intent)</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>月搜量 (Volume)</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>KD (难度)</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>CPC ($)</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Google Trends 飙升信号</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>SERP 盘面真实情况</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>市场缺口类型</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>终审判定</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>立项理由与推荐方案</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>2048 cupcakes</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>休闲数字/消除变体网页游戏 (Cupcake 甜点主题 2048)</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>201000</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>长期常青稳居高搜量，无明显衰退</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>头部为 2048cupcakes.net 与老旧聚合页，充斥大面积弹窗广告、加载缓慢且移动端无触控自适应</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>质量与体验缺口 (老旧站点广告多、移动端体验极差)</t>
+        </is>
+      </c>
+      <c r="I2" s="10" t="inlineStr">
+        <is>
+          <t>立项 (S级强推)</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>基于 MIT 开源 2048 引擎，替换精美高分辨率甜品 SVG/PNG 图标；零广告秒开，搜量超 20 万且 KD 为 0，极速冲上首屏</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>coreball</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>敏捷反应/穿针引线插针小游戏 (Coreball / AA 变体)</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>165000</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>稳步攀升，长尾 coreball unblocked 搜索量大增</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Arealme (广告繁杂阻碍视线)、Hooda Math、多个非官方聚合镜像，体验臃肿</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>独立微端与形态缺口 (缺乏零广告、暗黑极简纯净独立微端)</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
+        <is>
+          <t>立项 (S级强推)</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>纯 Canvas 2D 绘制旋转中枢与飞针，代码量 &lt;300 行；极简深色模式、零延迟秒开，支持键盘空格与触屏点击，精准满足校园/摸鱼需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>spacebar clicker</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>键盘连击/放置增量小游戏 (Spacebar Clicker)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>246000</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>校园学生端常青高搜量，工作日高峰特征明显</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Poki、cpstest.org、hoodamath，大部分为早期粗糙版本或单纯连击测速器，缺乏增量升级深度</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>体验缺口与校园连通缺口 (缺乏现代霓虹科技风增量成长反馈与 Chromebook 优化)</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>立项 (S级强推)</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>结合极简键盘敲击与放置自动化升级树（猴子按键、火箭推力、AI托管），玩家粘性极高，留存时长惊人</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>puppet hockey</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>双人/单人 1v1 大头冰球街机对战游戏</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>90500</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>长期稳定高搜量，怀旧街机搜索群稳定</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>大量原 Flash 站点因 Flash 停运损坏 (Ruffle 报错/黑屏)，聚合站加载失败率高</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>技术断层缺口 (Flash 淘汰后原生 HTML5 供给严重匮乏)</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>立项 (A级蓝海)</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>经典大头人偶物理跳跃与击球，KD 仅为 0！轻量 2D 物理引擎重构 HTML5 原生版，直接收割 9 万搜量断层流量</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>snow rider 3d unblocked</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>3D 无尽雪橇滑雪跑酷网页游戏 (学校无限制版)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>90500</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>季节性高热度 + 校园端突破网络限制搜索</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>各类 GitHub IO / Google Sites 镜像站，但资源包高达 30MB，低配设备加载极慢且易崩溃</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>性能与网络连通缺口 (极速 CDN、轻量化资源包、防封锁架构)</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>立项 (高变现 A级)</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>CPC 高达 .49，商业价值极高；针对海外学生群体打造零延迟秒开 3D 跑酷，轻量化资源包保障 Chromebook 流畅 60fps</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>brainrot clicker</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>梗文化/放置连点器微端 (Skibidi/Sigma/Rizz 梗题材)</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>49500</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>2026 全球年轻人/学生群体病毒式飙升词</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>头部仅个别 Scratch 粗糙移植版，缺乏成熟独立 Web 应用</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>内容与文化缺口 (极速爆发的 Gen-Z 梗文化无专业游戏承接)</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>立项 (高传播 A级)</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>纯前端 DOM + 音效触发，开发门槛极低；病毒传播能力极强，极易在 TikTok/Reddit 引发自然外链</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>feetle</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>每日单词阶梯谜题 (Word Ladder 变体)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>8500</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>+23,500% 突发爆发 (Google Trends 突发飙升榜首)</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>仅有官方 feetle.fun (每日仅1题)，搜索中大量出现 feetle unlimited / practice</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>模式缺口 (无限答题与题库归档缺口，同 Costcodle Unlimited 逻辑)</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>立项 (新词蓝海)</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>每次换1个字母将起始词变为 FEET；利用静态字典树 BFS 自动生成无限题库，做 Feetle Unlimited 降维截流</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>universal paperclips</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>哲学/AI 增量放置模拟神作 (Universal Paperclips)</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>+17,850% 爆发飙升 (AI 圈与社交媒体二次走红)</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>原作者 2017 年纯 HTML 页面排 #1，但排版陈旧无暗黑模式，手机端完全无法正常触控缩放</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>移动端触控与现代化 UI 缺口 (排版过时、字体极小、缺少现代响应式与深色模式)</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>立项 (经典长青 A级)</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>基于 MIT 开源逻辑重构现代化 UI，加入深色质感排版与移动端触控适配，大幅提升留存</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>candy clicker</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>休闲糖果消除/放置小游戏</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>40500</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>长年稳定搜索</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>聚合页嵌入，广告繁琐，加载较慢</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>极简形态缺口 (纯净微端)</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>立项 (B级 极低成本)</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>单日即可手搓完成的纯静态放置小游戏，作为游戏矩阵的轻量长尾节点</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>thorn and balloons</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>物理碰撞/弹射刺球消除气球益智解谜</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>40500</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>搜索稳定，移动端衍生流量大</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>前排多为 Google Play / App Store 移动端下载链接，缺少直接免下载网页版</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>终端与载体缺口 (手游向 Web 即玩端的移植缺口)</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>立项 (B级)</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>桌面端用户不想下载模拟器，纯 Canvas 2D 物理反弹关卡即可精准满足即玩需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>low's adventure 3</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>复古像素横版平台闯关游戏 (Low's Adventures)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>74000</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>稳定高搜量，系列作品人气高</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Hooda Math、CrazyGames 聚合分发，无独立官网</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>品牌独立站与关卡全集缺口</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>观察 (A级储备)</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>搜量高达 74k 且 KD 为 0，但关卡地图制作量较大，适合作为矩阵第二梯队关卡储备</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>rodha</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>极简几何平台跳跃跑酷</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>110000</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>稳中有升，平台跳跃受众稳定</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>CrazyGames / Coolmathgames 托管，无独立专用站点</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>独立微端与无障碍极速版缺口</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>观察 (A级储备)</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>搜量突破 11 万且 KD 仅 6，对物理手感调教要求较高，适合后续扩充</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>ovo unblocked</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>火柴人跑酷/极速微冲刺闯关游戏 (OvO Stickman Parkour)</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>60500</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>校园学生端长期常青，搜量极其稳定 (主词 ovo game 搜量 24.6 万)</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>大量旧 Google Sites 镜像失效或被学校封锁，缺少高质量独立秒开站点</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>网络连通与独立微端缺口</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>立项 (S级强推)</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>纯 HTML5/JS 物理平台跳跃，支持滑动、蹬墙跳、下砸蓄力，内置计时器与关卡存档，精准收割校园流量</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>drift boss</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>单键极简视角屋顶漂移避障游戏 (Drift Boss)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>165000</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>稳定高频搜索，学生白领摸鱼高发</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>头部为 Coolmathgames、MathPlayground 聚合分发，广告繁多且有不可跳过贴片</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>极简形态与纯净微端缺口</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>立项 (S级强推)</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>核心操作仅需长按右转/松开左转，单键物理机制极易开发；纯静态 Canvas 2D/3D，加入车辆皮肤与本地解锁成长</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>electron dash</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>3D 霓虹旋转管道无尽奔跑避障 (Run 3 玩法精神续作)</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>110000</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>搜索量持续稳中有升，无官方截流</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>聚合平台内嵌，加载资源包偏大且常被防火墙屏蔽</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>极速 CDN 性能与校园连通缺口</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>立项 (高变现 A级)</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>轻量 Three.js/WebGL 管道生成算法，控制包体在 2MB 内，CPC 高达 .50，学生端变现利器</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>planet clicker</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>太空星球殖民/能量开采放置连点器 (Planet Clicker)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>135000</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>常年高搜量，放置挂机类核心词</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>前排多为 Scratch 粗糙移植版，全屏适配差且无法离线保存</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>体验与技术缺口 (老旧 Scratch 移植版体验糟糕)</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>立项 (A级 休闲放置)</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>纯 DOM/SVG 现代化深色宇宙重构，加入地球/火星/金星自动化科技树与本地持久化存档，留存时长极佳</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>tunnel rush unblocked</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>3D 第一人称致幻极速隧道闪避 (Tunnel Rush)</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Google Trends 突发上升 +140% 飙升 (主词搜量 &gt;30 万)</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>充斥各种 66ez 等老旧镜像站，30 秒不可跳过视频广告泛滥</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>质量与纯净度缺口 (广告侵扰严重、加载慢)</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>立项 (A级 极速跑酷)</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>纯前端 WebGL 隧道程序化生成，零广告即开即玩，手感丝滑秒杀劣质镜像</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>head soccer 2026</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>1v1 大头人偶足球物理对抗小游戏 (Head Soccer)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>33100</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>搜索稳定，大头体育系列受众庞大且 KD 为 0</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>缺乏独立垂直站，多为 Flash 损坏或老旧模拟器</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>技术断层缺口 (Flash 淘汰原生重构)</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>立项 (A级 零成本代码复用)</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>完全复用 puppet hockey 的 2D 物理碰撞引擎，仅替换球体与角色贴图，即可 1 天内双发两款爆款站</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>acceleration city</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>3D 霓虹赛车特技与赛道编辑小游戏</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>368000</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>超高搜量 (36.8 万) 且 KD 为 0，无任何官方垄断</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>仅散落于教育机构页面（如 CS2N/CMU），缺乏独立商业化专精站点</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>独立品牌站缺口</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>立项 (高搜量 A级)</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>极低多边形 3D 赛车特技跑酷，满足桌面端极速畅玩需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>drift hunters unblocked</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>3D 拟真漂移调车沙盒游戏</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>33100</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>校园高频突破限制搜索，CPC 达 .82</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>GitHub IO 与 Google Sites 镜像站并存，加载较重</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>性能与防封锁镜像缺口</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>立项 (B级 需轻量化)</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>优化 WebGL 汽车物理材质，提供低配轻量模式供 Chromebook 极速运行</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>